<commit_message>
feat: add Lab 5 sample files for Claude Cowork path
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample-files/lab-2/bank_demo.xlsx
+++ b/sample-files/lab-2/bank_demo.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Accounts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Transactions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,10 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="MM/DD/YYYY"/>
+    <numFmt numFmtId="165" formatCode="MM/DD/YYYY"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -76,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -87,7 +86,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -516,6 +516,97 @@
       <c r="B8" s="4">
         <f>COUNTA(Transactions!A2:A51)</f>
         <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Rewards Program Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bronze Tier Accounts</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Silver Tier Accounts</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Gold Tier Accounts</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Avg Points - Bronze</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Avg Points - Silver</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Avg Points - Gold</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>8117</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Redemption Rate (18-29)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Redemption Rate (60+)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>8%</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -529,7 +620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -565,6 +656,21 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Age Segment</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Tier Level</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Rewards Points Balance</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -590,6 +696,19 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>18-29</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Bronze</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>1200</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -615,6 +734,19 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>45-59</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>8750</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -640,6 +772,19 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>30-44</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>4300</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -665,6 +810,19 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>60+</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Bronze</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>500</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -690,6 +848,19 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>30-44</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>9200</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -715,6 +886,19 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>18-29</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>3100</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -740,6 +924,19 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>60+</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>2800</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -765,6 +962,19 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>45-59</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Bronze</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>650</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -790,6 +1000,19 @@
           <t>Active</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>30-44</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Bronze</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>1100</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -814,6 +1037,19 @@
         <is>
           <t>Active</t>
         </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>18-29</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>6400</v>
       </c>
     </row>
   </sheetData>
@@ -827,7 +1063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -875,6 +1111,16 @@
           <t>Balance After</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Rewards Points Earned</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Redemption Flag</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -887,7 +1133,7 @@
           <t>ACC001</t>
         </is>
       </c>
-      <c r="C2" s="8" t="n">
+      <c r="C2" s="9" t="n">
         <v>46054</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -903,7 +1149,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -916,7 +1169,7 @@
           <t>ACC002</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="C3" s="9" t="n">
         <v>46055</v>
       </c>
       <c r="D3" t="inlineStr">
@@ -932,7 +1185,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -945,7 +1205,7 @@
           <t>ACC003</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="9" t="n">
         <v>46056</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -961,7 +1221,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>70</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -974,7 +1241,7 @@
           <t>ACC004</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n">
+      <c r="C5" s="9" t="n">
         <v>46057</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -990,7 +1257,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1003,7 +1277,7 @@
           <t>ACC005</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="9" t="n">
         <v>46058</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -1019,7 +1293,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1032,7 +1313,7 @@
           <t>ACC006</t>
         </is>
       </c>
-      <c r="C7" s="8" t="n">
+      <c r="C7" s="9" t="n">
         <v>46059</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -1048,7 +1329,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1061,7 +1349,7 @@
           <t>ACC007</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="9" t="n">
         <v>46060</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -1077,7 +1365,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>15</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1090,7 +1385,7 @@
           <t>ACC008</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="9" t="n">
         <v>46061</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -1106,7 +1401,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1119,7 +1421,7 @@
           <t>ACC009</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="9" t="n">
         <v>46062</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -1135,7 +1437,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1148,7 +1457,7 @@
           <t>ACC010</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="9" t="n">
         <v>46063</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -1164,7 +1473,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>15</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1177,7 +1493,7 @@
           <t>ACC001</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="9" t="n">
         <v>46064</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -1193,7 +1509,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1206,7 +1529,7 @@
           <t>ACC002</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="9" t="n">
         <v>46065</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -1222,7 +1545,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>105</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1235,7 +1565,7 @@
           <t>ACC003</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="9" t="n">
         <v>46066</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -1251,7 +1581,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1264,7 +1601,7 @@
           <t>ACC004</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="9" t="n">
         <v>46067</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -1280,7 +1617,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>10</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1293,7 +1637,7 @@
           <t>ACC005</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="9" t="n">
         <v>46068</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -1309,7 +1653,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1322,7 +1673,7 @@
           <t>ACC006</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="9" t="n">
         <v>46069</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -1338,7 +1689,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>15</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1351,7 +1709,7 @@
           <t>ACC007</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="9" t="n">
         <v>46070</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -1367,7 +1725,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1380,7 +1745,7 @@
           <t>ACC008</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="9" t="n">
         <v>46071</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -1396,7 +1761,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1409,7 +1781,7 @@
           <t>ACC009</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="9" t="n">
         <v>46072</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -1425,7 +1797,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1438,7 +1817,7 @@
           <t>ACC010</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="9" t="n">
         <v>46073</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -1454,7 +1833,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1467,7 +1853,7 @@
           <t>ACC001</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n">
+      <c r="C22" s="9" t="n">
         <v>46074</v>
       </c>
       <c r="D22" t="inlineStr">
@@ -1483,7 +1869,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>35</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1496,7 +1889,7 @@
           <t>ACC002</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n">
+      <c r="C23" s="9" t="n">
         <v>46075</v>
       </c>
       <c r="D23" t="inlineStr">
@@ -1512,7 +1905,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1525,7 +1925,7 @@
           <t>ACC003</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n">
+      <c r="C24" s="9" t="n">
         <v>46076</v>
       </c>
       <c r="D24" t="inlineStr">
@@ -1541,7 +1941,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>20</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1554,7 +1961,7 @@
           <t>ACC004</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n">
+      <c r="C25" s="9" t="n">
         <v>46077</v>
       </c>
       <c r="D25" t="inlineStr">
@@ -1570,7 +1977,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1583,7 +1997,7 @@
           <t>ACC005</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n">
+      <c r="C26" s="9" t="n">
         <v>46078</v>
       </c>
       <c r="D26" t="inlineStr">
@@ -1599,7 +2013,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>22</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1612,7 +2033,7 @@
           <t>ACC006</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n">
+      <c r="C27" s="9" t="n">
         <v>46079</v>
       </c>
       <c r="D27" t="inlineStr">
@@ -1628,7 +2049,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1641,7 +2069,7 @@
           <t>ACC007</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n">
+      <c r="C28" s="9" t="n">
         <v>46080</v>
       </c>
       <c r="D28" t="inlineStr">
@@ -1657,7 +2085,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1670,7 +2105,7 @@
           <t>ACC008</t>
         </is>
       </c>
-      <c r="C29" s="8" t="n">
+      <c r="C29" s="9" t="n">
         <v>46081</v>
       </c>
       <c r="D29" t="inlineStr">
@@ -1686,7 +2121,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>5</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1699,7 +2141,7 @@
           <t>ACC009</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n">
+      <c r="C30" s="9" t="n">
         <v>46082</v>
       </c>
       <c r="D30" t="inlineStr">
@@ -1715,7 +2157,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1728,7 +2177,7 @@
           <t>ACC010</t>
         </is>
       </c>
-      <c r="C31" s="8" t="n">
+      <c r="C31" s="9" t="n">
         <v>46083</v>
       </c>
       <c r="D31" t="inlineStr">
@@ -1744,7 +2193,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>105</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1757,7 +2213,7 @@
           <t>ACC001</t>
         </is>
       </c>
-      <c r="C32" s="8" t="n">
+      <c r="C32" s="9" t="n">
         <v>46084</v>
       </c>
       <c r="D32" t="inlineStr">
@@ -1773,7 +2229,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1786,7 +2249,7 @@
           <t>ACC002</t>
         </is>
       </c>
-      <c r="C33" s="8" t="n">
+      <c r="C33" s="9" t="n">
         <v>46085</v>
       </c>
       <c r="D33" t="inlineStr">
@@ -1802,7 +2265,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>30</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1815,7 +2285,7 @@
           <t>ACC003</t>
         </is>
       </c>
-      <c r="C34" s="8" t="n">
+      <c r="C34" s="9" t="n">
         <v>46086</v>
       </c>
       <c r="D34" t="inlineStr">
@@ -1831,7 +2301,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1844,7 +2321,7 @@
           <t>ACC004</t>
         </is>
       </c>
-      <c r="C35" s="8" t="n">
+      <c r="C35" s="9" t="n">
         <v>46087</v>
       </c>
       <c r="D35" t="inlineStr">
@@ -1860,7 +2337,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>7</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1873,7 +2357,7 @@
           <t>ACC005</t>
         </is>
       </c>
-      <c r="C36" s="8" t="n">
+      <c r="C36" s="9" t="n">
         <v>46088</v>
       </c>
       <c r="D36" t="inlineStr">
@@ -1889,7 +2373,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1902,7 +2393,7 @@
           <t>ACC006</t>
         </is>
       </c>
-      <c r="C37" s="8" t="n">
+      <c r="C37" s="9" t="n">
         <v>46089</v>
       </c>
       <c r="D37" t="inlineStr">
@@ -1918,7 +2409,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1931,7 +2429,7 @@
           <t>ACC007</t>
         </is>
       </c>
-      <c r="C38" s="8" t="n">
+      <c r="C38" s="9" t="n">
         <v>46090</v>
       </c>
       <c r="D38" t="inlineStr">
@@ -1947,7 +2445,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="n">
+        <v>10</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1960,7 +2465,7 @@
           <t>ACC008</t>
         </is>
       </c>
-      <c r="C39" s="8" t="n">
+      <c r="C39" s="9" t="n">
         <v>46091</v>
       </c>
       <c r="D39" t="inlineStr">
@@ -1976,7 +2481,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1989,7 +2501,7 @@
           <t>ACC009</t>
         </is>
       </c>
-      <c r="C40" s="8" t="n">
+      <c r="C40" s="9" t="n">
         <v>46092</v>
       </c>
       <c r="D40" t="inlineStr">
@@ -2005,7 +2517,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>35</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2018,7 +2537,7 @@
           <t>ACC010</t>
         </is>
       </c>
-      <c r="C41" s="8" t="n">
+      <c r="C41" s="9" t="n">
         <v>46093</v>
       </c>
       <c r="D41" t="inlineStr">
@@ -2034,7 +2553,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2047,7 +2573,7 @@
           <t>ACC001</t>
         </is>
       </c>
-      <c r="C42" s="8" t="n">
+      <c r="C42" s="9" t="n">
         <v>46094</v>
       </c>
       <c r="D42" t="inlineStr">
@@ -2063,7 +2589,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="n">
+        <v>10</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2076,7 +2609,7 @@
           <t>ACC002</t>
         </is>
       </c>
-      <c r="C43" s="8" t="n">
+      <c r="C43" s="9" t="n">
         <v>46095</v>
       </c>
       <c r="D43" t="inlineStr">
@@ -2092,7 +2625,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2105,7 +2645,7 @@
           <t>ACC003</t>
         </is>
       </c>
-      <c r="C44" s="8" t="n">
+      <c r="C44" s="9" t="n">
         <v>46096</v>
       </c>
       <c r="D44" t="inlineStr">
@@ -2121,7 +2661,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="n">
+        <v>15</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2134,7 +2681,7 @@
           <t>ACC004</t>
         </is>
       </c>
-      <c r="C45" s="8" t="n">
+      <c r="C45" s="9" t="n">
         <v>46097</v>
       </c>
       <c r="D45" t="inlineStr">
@@ -2150,7 +2697,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2163,7 +2717,7 @@
           <t>ACC005</t>
         </is>
       </c>
-      <c r="C46" s="8" t="n">
+      <c r="C46" s="9" t="n">
         <v>46098</v>
       </c>
       <c r="D46" t="inlineStr">
@@ -2179,7 +2733,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2192,7 +2753,7 @@
           <t>ACC006</t>
         </is>
       </c>
-      <c r="C47" s="8" t="n">
+      <c r="C47" s="9" t="n">
         <v>46099</v>
       </c>
       <c r="D47" t="inlineStr">
@@ -2208,7 +2769,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="n">
+        <v>10</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2221,7 +2789,7 @@
           <t>ACC007</t>
         </is>
       </c>
-      <c r="C48" s="8" t="n">
+      <c r="C48" s="9" t="n">
         <v>46100</v>
       </c>
       <c r="D48" t="inlineStr">
@@ -2237,7 +2805,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2250,7 +2825,7 @@
           <t>ACC008</t>
         </is>
       </c>
-      <c r="C49" s="8" t="n">
+      <c r="C49" s="9" t="n">
         <v>46101</v>
       </c>
       <c r="D49" t="inlineStr">
@@ -2266,7 +2841,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>35</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2279,7 +2861,7 @@
           <t>ACC009</t>
         </is>
       </c>
-      <c r="C50" s="8" t="n">
+      <c r="C50" s="9" t="n">
         <v>46102</v>
       </c>
       <c r="D50" t="inlineStr">
@@ -2295,7 +2877,14 @@
           <t>Withdrawal</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2308,7 +2897,7 @@
           <t>ACC010</t>
         </is>
       </c>
-      <c r="C51" s="8" t="n">
+      <c r="C51" s="9" t="n">
         <v>46103</v>
       </c>
       <c r="D51" t="inlineStr">
@@ -2324,7 +2913,14 @@
           <t>Deposit</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="n">
+        <v>30</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>